<commit_message>
feat(panel): aplica el bucle de fortalecimiento (convergió en 2 vueltas)
- Reaplica en las capas lo que la réplica cambió: 10 clases del contraste de
  2.°–8.°, 7 elementos de contenido de 7.° y 9.°, 1 decisión y 1 asignación;
  la solidez queda en 415 registros del panel.
- Decisión delegada (verificada en la fuente): fuerzas intermoleculares pasan
  a «sin referente» (solo ENG GCSE p. 20; HK p. 81 es Extension Part).
- Una asignación rechazada queda como observación del elemento, no de toda la
  división; el CSV de asignaciones trae su estado.
- Contraste de 2.°–8.° reconstruido: potencia eléctrica y leyes de los gases
  dejan de ser tardías; mitosis y capas de la atmósfera, adelantadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/2_8/Contraste_quimica.xlsx
+++ b/internacional/2_8/Contraste_quimica.xlsx
@@ -1044,7 +1044,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fuerzas intermoleculares y propiedades físicas</t>
+          <t>Iones</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1053,10 +1053,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
         <v>8</v>
@@ -1064,7 +1064,16 @@
       <c r="G8" t="n">
         <v>8.5</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
+        <v>8</v>
+      </c>
+      <c r="J8" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M8" t="n">
         <v>7</v>
       </c>
       <c r="O8" t="n">
@@ -1073,30 +1082,36 @@
       <c r="P8" t="n">
         <v>1</v>
       </c>
-      <c r="Q8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z8" t="n">
+      <c r="R8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V8" t="n">
         <v>1</v>
       </c>
       <c r="AF8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>posterior</t>
+          <t>adelantado</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Iones</t>
+          <t>Masa atómica relativa</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1110,40 +1125,25 @@
       <c r="D9" t="n">
         <v>5</v>
       </c>
-      <c r="F9" t="n">
-        <v>8</v>
-      </c>
       <c r="G9" t="n">
         <v>8.5</v>
       </c>
-      <c r="I9" t="n">
-        <v>8</v>
-      </c>
-      <c r="J9" t="n">
-        <v>7</v>
-      </c>
       <c r="L9" t="n">
         <v>7.5</v>
       </c>
       <c r="M9" t="n">
         <v>7</v>
       </c>
-      <c r="O9" t="n">
-        <v>1</v>
-      </c>
       <c r="P9" t="n">
         <v>1</v>
       </c>
-      <c r="R9" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" t="n">
-        <v>1</v>
-      </c>
       <c r="U9" t="n">
         <v>1</v>
       </c>
       <c r="V9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z9" t="n">
         <v>1</v>
       </c>
       <c r="AF9" t="n">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
@@ -1163,7 +1163,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Masa atómica relativa</t>
+          <t>Reutilización y reciclaje de materiales</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1172,13 +1172,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>8.5</v>
+        <v>6</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4</v>
       </c>
       <c r="L10" t="n">
         <v>7.5</v>
@@ -1186,9 +1198,21 @@
       <c r="M10" t="n">
         <v>7</v>
       </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
       <c r="P10" t="n">
         <v>1</v>
       </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1</v>
+      </c>
       <c r="U10" t="n">
         <v>1</v>
       </c>
@@ -1199,11 +1223,11 @@
         <v>1</v>
       </c>
       <c r="AF10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>adelantado</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
@@ -1215,7 +1239,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Reutilización y reciclaje de materiales</t>
+          <t>Mezclas homogéneas y heterogéneas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1229,26 +1253,35 @@
       <c r="D11" t="n">
         <v>2</v>
       </c>
+      <c r="E11" t="n">
+        <v>6</v>
+      </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="n">
         <v>6</v>
-      </c>
-      <c r="H11" t="n">
-        <v>7</v>
       </c>
       <c r="J11" t="n">
         <v>4.5</v>
       </c>
       <c r="K11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L11" t="n">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="M11" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
       </c>
       <c r="O11" t="n">
         <v>1</v>
@@ -1257,6 +1290,9 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
@@ -1291,7 +1327,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mezclas homogéneas y heterogéneas</t>
+          <t>Evolución de los modelos atómicos</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1300,70 +1336,43 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" t="n">
         <v>6</v>
       </c>
-      <c r="F12" t="n">
+      <c r="K12" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF12" t="n">
         <v>5</v>
-      </c>
-      <c r="G12" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I12" t="n">
-        <v>6</v>
-      </c>
-      <c r="J12" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K12" t="n">
-        <v>6</v>
-      </c>
-      <c r="L12" t="n">
-        <v>5</v>
-      </c>
-      <c r="M12" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="N12" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" t="n">
-        <v>1</v>
-      </c>
-      <c r="P12" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>1</v>
-      </c>
-      <c r="R12" t="n">
-        <v>1</v>
-      </c>
-      <c r="S12" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" t="n">
-        <v>1</v>
-      </c>
-      <c r="U12" t="n">
-        <v>1</v>
-      </c>
-      <c r="V12" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF12" t="n">
-        <v>2</v>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
@@ -1379,7 +1388,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Evolución de los modelos atómicos</t>
+          <t>Moléculas y fórmulas químicas</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1394,13 +1403,25 @@
         <v>5</v>
       </c>
       <c r="E13" t="n">
+        <v>7</v>
+      </c>
+      <c r="F13" t="n">
         <v>8</v>
       </c>
       <c r="G13" t="n">
         <v>6</v>
       </c>
+      <c r="H13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" t="n">
+        <v>7</v>
+      </c>
       <c r="K13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L13" t="n">
         <v>7.5</v>
@@ -1411,9 +1432,21 @@
       <c r="N13" t="n">
         <v>1</v>
       </c>
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
       <c r="P13" t="n">
         <v>1</v>
       </c>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1</v>
+      </c>
       <c r="T13" t="n">
         <v>1</v>
       </c>
@@ -1421,6 +1454,9 @@
         <v>1</v>
       </c>
       <c r="V13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z13" t="n">
         <v>1</v>
       </c>
       <c r="AF13" t="n">
@@ -1440,7 +1476,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Moléculas y fórmulas químicas</t>
+          <t>Propiedades periódicas</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1454,55 +1490,19 @@
       <c r="D14" t="n">
         <v>5</v>
       </c>
-      <c r="E14" t="n">
-        <v>7</v>
-      </c>
-      <c r="F14" t="n">
-        <v>8</v>
-      </c>
       <c r="G14" t="n">
         <v>6</v>
       </c>
-      <c r="H14" t="n">
-        <v>7</v>
-      </c>
-      <c r="I14" t="n">
-        <v>7</v>
-      </c>
-      <c r="J14" t="n">
-        <v>7</v>
-      </c>
       <c r="K14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L14" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="M14" t="n">
         <v>7</v>
       </c>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
-        <v>1</v>
-      </c>
       <c r="P14" t="n">
         <v>1</v>
       </c>
-      <c r="Q14" t="n">
-        <v>1</v>
-      </c>
-      <c r="R14" t="n">
-        <v>1</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1</v>
-      </c>
       <c r="T14" t="n">
-        <v>1</v>
-      </c>
-      <c r="U14" t="n">
         <v>1</v>
       </c>
       <c r="V14" t="n">
@@ -1528,7 +1528,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Propiedades periódicas</t>
+          <t>Propiedades singulares del agua</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1537,34 +1537,43 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="n">
         <v>5</v>
       </c>
       <c r="G15" t="n">
         <v>6</v>
       </c>
+      <c r="H15" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
       <c r="K15" t="n">
-        <v>8</v>
-      </c>
-      <c r="M15" t="n">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
       </c>
       <c r="P15" t="n">
         <v>1</v>
       </c>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
       <c r="T15" t="n">
         <v>1</v>
       </c>
-      <c r="V15" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>1</v>
-      </c>
       <c r="AF15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
@@ -1580,7 +1589,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Propiedades singulares del agua</t>
+          <t>Química descriptiva de los elementos</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1589,43 +1598,40 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>7</v>
+      </c>
+      <c r="M16" t="n">
+        <v>7</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF16" t="n">
         <v>5</v>
-      </c>
-      <c r="G16" t="n">
-        <v>6</v>
-      </c>
-      <c r="H16" t="n">
-        <v>7</v>
-      </c>
-      <c r="I16" t="n">
-        <v>3</v>
-      </c>
-      <c r="K16" t="n">
-        <v>6</v>
-      </c>
-      <c r="O16" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>1</v>
-      </c>
-      <c r="R16" t="n">
-        <v>1</v>
-      </c>
-      <c r="T16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>3</v>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
@@ -1641,7 +1647,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Química descriptiva de los elementos</t>
+          <t>Reacción química y sus evidencias</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1650,22 +1656,40 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="n">
         <v>5</v>
       </c>
       <c r="F17" t="n">
         <v>8</v>
       </c>
       <c r="G17" t="n">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="H17" t="n">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5</v>
+      </c>
+      <c r="J17" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" t="n">
+        <v>7.5</v>
       </c>
       <c r="M17" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
       </c>
       <c r="O17" t="n">
         <v>1</v>
@@ -1676,14 +1700,23 @@
       <c r="Q17" t="n">
         <v>1</v>
       </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" t="n">
+        <v>1</v>
+      </c>
       <c r="V17" t="n">
         <v>1</v>
       </c>
-      <c r="Z17" t="n">
-        <v>1</v>
-      </c>
       <c r="AF17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
@@ -1699,7 +1732,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Reacción química y sus evidencias</t>
+          <t>Métodos físicos de separación de mezclas</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1714,31 +1747,31 @@
         <v>2</v>
       </c>
       <c r="E18" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" t="n">
         <v>5</v>
-      </c>
-      <c r="F18" t="n">
-        <v>8</v>
       </c>
       <c r="G18" t="n">
         <v>3</v>
       </c>
       <c r="H18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J18" t="n">
         <v>4.5</v>
       </c>
       <c r="K18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L18" t="n">
         <v>7.5</v>
       </c>
       <c r="M18" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="N18" t="n">
         <v>1</v>
@@ -1765,6 +1798,9 @@
         <v>1</v>
       </c>
       <c r="V18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z18" t="n">
         <v>1</v>
       </c>
       <c r="AF18" t="n">
@@ -1784,7 +1820,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Métodos físicos de separación de mezclas</t>
+          <t>Solubilidad y disoluciones saturadas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1793,16 +1829,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G19" t="n">
         <v>3</v>
@@ -1825,9 +1858,6 @@
       <c r="M19" t="n">
         <v>2.5</v>
       </c>
-      <c r="N19" t="n">
-        <v>1</v>
-      </c>
       <c r="O19" t="n">
         <v>1</v>
       </c>
@@ -1852,11 +1882,8 @@
       <c r="V19" t="n">
         <v>1</v>
       </c>
-      <c r="Z19" t="n">
-        <v>1</v>
-      </c>
       <c r="AF19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
@@ -1865,14 +1892,14 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Solubilidad y disoluciones saturadas</t>
+          <t>Organización de la tabla periódica</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1881,34 +1908,31 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
         <v>8</v>
       </c>
       <c r="G20" t="n">
+        <v>6</v>
+      </c>
+      <c r="H20" t="n">
         <v>3</v>
       </c>
-      <c r="H20" t="n">
-        <v>2</v>
-      </c>
-      <c r="I20" t="n">
-        <v>4</v>
-      </c>
       <c r="J20" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="K20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L20" t="n">
         <v>7.5</v>
       </c>
       <c r="M20" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="O20" t="n">
         <v>1</v>
@@ -1919,9 +1943,6 @@
       <c r="Q20" t="n">
         <v>1</v>
       </c>
-      <c r="R20" t="n">
-        <v>1</v>
-      </c>
       <c r="S20" t="n">
         <v>1</v>
       </c>
@@ -1934,8 +1955,11 @@
       <c r="V20" t="n">
         <v>1</v>
       </c>
+      <c r="Z20" t="n">
+        <v>1</v>
+      </c>
       <c r="AF20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
@@ -1944,14 +1968,14 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>adelantado</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Organización de la tabla periódica</t>
+          <t>Calidad y tratamiento del agua</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1960,58 +1984,49 @@
         </is>
       </c>
       <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" t="n">
         <v>5</v>
       </c>
-      <c r="D21" t="n">
+      <c r="G21" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" t="n">
+        <v>7</v>
+      </c>
+      <c r="L21" t="n">
         <v>5</v>
       </c>
-      <c r="F21" t="n">
-        <v>8</v>
-      </c>
-      <c r="G21" t="n">
-        <v>6</v>
-      </c>
-      <c r="H21" t="n">
+      <c r="M21" t="n">
+        <v>7</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
+      <c r="T21" t="n">
+        <v>1</v>
+      </c>
+      <c r="U21" t="n">
+        <v>1</v>
+      </c>
+      <c r="V21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF21" t="n">
         <v>3</v>
-      </c>
-      <c r="J21" t="n">
-        <v>7</v>
-      </c>
-      <c r="K21" t="n">
-        <v>8</v>
-      </c>
-      <c r="L21" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="M21" t="n">
-        <v>7</v>
-      </c>
-      <c r="O21" t="n">
-        <v>1</v>
-      </c>
-      <c r="P21" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>1</v>
-      </c>
-      <c r="S21" t="n">
-        <v>1</v>
-      </c>
-      <c r="T21" t="n">
-        <v>1</v>
-      </c>
-      <c r="U21" t="n">
-        <v>1</v>
-      </c>
-      <c r="V21" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF21" t="n">
-        <v>5</v>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
@@ -2027,37 +2042,40 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Calidad y tratamiento del agua</t>
+          <t>Ácidos y bases: propiedades</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G22" t="n">
+        <v>6</v>
+      </c>
+      <c r="H22" t="n">
+        <v>7</v>
+      </c>
+      <c r="I22" t="n">
         <v>5</v>
       </c>
-      <c r="G22" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H22" t="n">
-        <v>2</v>
-      </c>
-      <c r="K22" t="n">
-        <v>7</v>
+      <c r="J22" t="n">
+        <v>4.5</v>
       </c>
       <c r="L22" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="M22" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="O22" t="n">
         <v>1</v>
@@ -2068,7 +2086,10 @@
       <c r="Q22" t="n">
         <v>1</v>
       </c>
-      <c r="T22" t="n">
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="n">
         <v>1</v>
       </c>
       <c r="U22" t="n">
@@ -2078,23 +2099,23 @@
         <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ácidos y bases: propiedades</t>
+          <t>Cambios de estado</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2103,32 +2124,41 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>8</v>
       </c>
       <c r="G23" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4</v>
       </c>
       <c r="L23" t="n">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="M23" t="n">
         <v>2.5</v>
       </c>
+      <c r="N23" t="n">
+        <v>1</v>
+      </c>
       <c r="O23" t="n">
         <v>1</v>
       </c>
@@ -2144,14 +2174,20 @@
       <c r="S23" t="n">
         <v>1</v>
       </c>
+      <c r="T23" t="n">
+        <v>1</v>
+      </c>
       <c r="U23" t="n">
         <v>1</v>
       </c>
       <c r="V23" t="n">
         <v>1</v>
       </c>
+      <c r="Z23" t="n">
+        <v>1</v>
+      </c>
       <c r="AF23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AG23" t="inlineStr">
         <is>
@@ -2167,7 +2203,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cambios de estado</t>
+          <t>Combustibles fósiles y biocombustibles</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2176,40 +2212,25 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
         <v>8</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
-      </c>
-      <c r="I24" t="n">
         <v>3</v>
-      </c>
-      <c r="J24" t="n">
-        <v>2.5</v>
       </c>
       <c r="K24" t="n">
         <v>4</v>
       </c>
-      <c r="L24" t="n">
-        <v>4</v>
-      </c>
       <c r="M24" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N24" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O24" t="n">
         <v>1</v>
@@ -2220,18 +2241,9 @@
       <c r="Q24" t="n">
         <v>1</v>
       </c>
-      <c r="R24" t="n">
-        <v>1</v>
-      </c>
-      <c r="S24" t="n">
-        <v>1</v>
-      </c>
       <c r="T24" t="n">
         <v>1</v>
       </c>
-      <c r="U24" t="n">
-        <v>1</v>
-      </c>
       <c r="V24" t="n">
         <v>1</v>
       </c>
@@ -2239,7 +2251,7 @@
         <v>1</v>
       </c>
       <c r="AF24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
@@ -2255,7 +2267,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Combustibles fósiles y biocombustibles</t>
+          <t>Combustión</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2268,21 +2280,33 @@
       </c>
       <c r="D25" t="n">
         <v>7</v>
+      </c>
+      <c r="E25" t="n">
+        <v>8</v>
       </c>
       <c r="F25" t="n">
         <v>8</v>
       </c>
       <c r="G25" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H25" t="n">
         <v>3</v>
       </c>
-      <c r="K25" t="n">
-        <v>4</v>
+      <c r="I25" t="n">
+        <v>5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L25" t="n">
+        <v>7.5</v>
       </c>
       <c r="M25" t="n">
-        <v>7</v>
+        <v>2.5</v>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
       </c>
       <c r="O25" t="n">
         <v>1</v>
@@ -2293,7 +2317,13 @@
       <c r="Q25" t="n">
         <v>1</v>
       </c>
-      <c r="T25" t="n">
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" t="n">
         <v>1</v>
       </c>
       <c r="V25" t="n">
@@ -2312,14 +2342,14 @@
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Combustión</t>
+          <t>Composición del aire y contaminantes atmosféricos</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2328,38 +2358,26 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>7</v>
-      </c>
-      <c r="E26" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>8</v>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
+        <v>8.5</v>
       </c>
       <c r="H26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
         <v>5</v>
       </c>
       <c r="J26" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L26" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="M26" t="n">
         <v>2.5</v>
       </c>
-      <c r="N26" t="n">
-        <v>1</v>
-      </c>
       <c r="O26" t="n">
         <v>1</v>
       </c>
@@ -2375,33 +2393,24 @@
       <c r="S26" t="n">
         <v>1</v>
       </c>
-      <c r="U26" t="n">
-        <v>1</v>
-      </c>
-      <c r="V26" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>1</v>
-      </c>
       <c r="AF26" t="n">
         <v>7</v>
       </c>
       <c r="AG26" t="inlineStr">
         <is>
+          <t>adelantado</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
           <t>alineado</t>
-        </is>
-      </c>
-      <c r="AH26" t="inlineStr">
-        <is>
-          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Composición del aire y contaminantes atmosféricos</t>
+          <t>Conservación de la masa</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2410,25 +2419,37 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>7</v>
+      </c>
+      <c r="E27" t="n">
+        <v>8</v>
       </c>
       <c r="F27" t="n">
         <v>8</v>
       </c>
       <c r="G27" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J27" t="n">
-        <v>2.5</v>
+        <v>7</v>
+      </c>
+      <c r="L27" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M27" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
       </c>
       <c r="O27" t="n">
         <v>1</v>
@@ -2445,24 +2466,30 @@
       <c r="S27" t="n">
         <v>1</v>
       </c>
+      <c r="U27" t="n">
+        <v>1</v>
+      </c>
+      <c r="V27" t="n">
+        <v>1</v>
+      </c>
       <c r="AF27" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>adelantado</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Conservación de la masa</t>
+          <t>Disolución y rapidez de disolución</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2471,40 +2498,31 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
-      </c>
-      <c r="E28" t="n">
-        <v>8</v>
-      </c>
-      <c r="F28" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G28" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H28" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I28" t="n">
         <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="K28" t="n">
+        <v>6</v>
       </c>
       <c r="L28" t="n">
         <v>7.5</v>
       </c>
       <c r="M28" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="N28" t="n">
-        <v>1</v>
-      </c>
-      <c r="O28" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="P28" t="n">
         <v>1</v>
@@ -2518,6 +2536,9 @@
       <c r="S28" t="n">
         <v>1</v>
       </c>
+      <c r="T28" t="n">
+        <v>1</v>
+      </c>
       <c r="U28" t="n">
         <v>1</v>
       </c>
@@ -2525,7 +2546,7 @@
         <v>1</v>
       </c>
       <c r="AF28" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AG28" t="inlineStr">
         <is>
@@ -2534,14 +2555,14 @@
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Disolución y rapidez de disolución</t>
+          <t>Ecuación química y su balanceo</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2550,31 +2571,40 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8</v>
+      </c>
+      <c r="F29" t="n">
+        <v>8</v>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I29" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J29" t="n">
         <v>4.5</v>
       </c>
-      <c r="K29" t="n">
-        <v>6</v>
-      </c>
       <c r="L29" t="n">
         <v>7.5</v>
       </c>
       <c r="M29" t="n">
-        <v>2.5</v>
+        <v>7</v>
+      </c>
+      <c r="N29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O29" t="n">
+        <v>1</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
@@ -2588,17 +2618,17 @@
       <c r="S29" t="n">
         <v>1</v>
       </c>
-      <c r="T29" t="n">
-        <v>1</v>
-      </c>
       <c r="U29" t="n">
         <v>1</v>
       </c>
       <c r="V29" t="n">
         <v>1</v>
       </c>
+      <c r="Z29" t="n">
+        <v>1</v>
+      </c>
       <c r="AF29" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AG29" t="inlineStr">
         <is>
@@ -2614,7 +2644,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ecuación química y su balanceo</t>
+          <t>Escala de pH</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2623,13 +2653,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" t="n">
         <v>8</v>
@@ -2641,7 +2668,7 @@
         <v>7</v>
       </c>
       <c r="I30" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J30" t="n">
         <v>4.5</v>
@@ -2650,10 +2677,7 @@
         <v>7.5</v>
       </c>
       <c r="M30" t="n">
-        <v>7</v>
-      </c>
-      <c r="N30" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="O30" t="n">
         <v>1</v>
@@ -2674,9 +2698,6 @@
         <v>1</v>
       </c>
       <c r="V30" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z30" t="n">
         <v>1</v>
       </c>
       <c r="AF30" t="n">
@@ -2696,7 +2717,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Escala de pH</t>
+          <t>Estados de la materia</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2705,31 +2726,40 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
       </c>
       <c r="F31" t="n">
         <v>8</v>
       </c>
       <c r="G31" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J31" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="K31" t="n">
+        <v>4</v>
       </c>
       <c r="L31" t="n">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="M31" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>1</v>
       </c>
       <c r="O31" t="n">
         <v>1</v>
@@ -2746,14 +2776,20 @@
       <c r="S31" t="n">
         <v>1</v>
       </c>
+      <c r="T31" t="n">
+        <v>1</v>
+      </c>
       <c r="U31" t="n">
         <v>1</v>
       </c>
       <c r="V31" t="n">
         <v>1</v>
       </c>
+      <c r="Z31" t="n">
+        <v>1</v>
+      </c>
       <c r="AF31" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AG31" t="inlineStr">
         <is>
@@ -2769,7 +2805,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Estados de la materia</t>
+          <t>Estequiometría</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2778,40 +2814,22 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F32" t="n">
         <v>8</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
-      </c>
-      <c r="H32" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="I32" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J32" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K32" t="n">
-        <v>4</v>
-      </c>
-      <c r="L32" t="n">
-        <v>4</v>
-      </c>
-      <c r="M32" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N32" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O32" t="n">
         <v>1</v>
@@ -2819,29 +2837,14 @@
       <c r="P32" t="n">
         <v>1</v>
       </c>
-      <c r="Q32" t="n">
-        <v>1</v>
-      </c>
       <c r="R32" t="n">
         <v>1</v>
       </c>
       <c r="S32" t="n">
         <v>1</v>
       </c>
-      <c r="T32" t="n">
-        <v>1</v>
-      </c>
-      <c r="U32" t="n">
-        <v>1</v>
-      </c>
-      <c r="V32" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z32" t="n">
-        <v>1</v>
-      </c>
       <c r="AF32" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AG32" t="inlineStr">
         <is>
@@ -2857,7 +2860,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Estequiometría</t>
+          <t>Indicadores ácido-base</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2866,22 +2869,25 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>8</v>
-      </c>
-      <c r="D33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F33" t="n">
         <v>8</v>
       </c>
       <c r="G33" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="I33" t="n">
+        <v>6</v>
+      </c>
+      <c r="H33" t="n">
         <v>7</v>
       </c>
       <c r="J33" t="n">
-        <v>7</v>
+        <v>4.5</v>
+      </c>
+      <c r="L33" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M33" t="n">
+        <v>2.5</v>
       </c>
       <c r="O33" t="n">
         <v>1</v>
@@ -2889,30 +2895,36 @@
       <c r="P33" t="n">
         <v>1</v>
       </c>
-      <c r="R33" t="n">
+      <c r="Q33" t="n">
         <v>1</v>
       </c>
       <c r="S33" t="n">
         <v>1</v>
       </c>
+      <c r="U33" t="n">
+        <v>1</v>
+      </c>
+      <c r="V33" t="n">
+        <v>1</v>
+      </c>
       <c r="AF33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AG33" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
       <c r="AH33" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>tardio</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Indicadores ácido-base</t>
+          <t>Materia y materiales</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2921,26 +2933,41 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>2</v>
+      </c>
+      <c r="D34" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2</v>
       </c>
       <c r="F34" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" t="n">
         <v>8</v>
       </c>
-      <c r="G34" t="n">
-        <v>6</v>
-      </c>
-      <c r="H34" t="n">
-        <v>7</v>
-      </c>
       <c r="J34" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="K34" t="n">
+        <v>4</v>
       </c>
       <c r="L34" t="n">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="M34" t="n">
         <v>2.5</v>
       </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
       <c r="O34" t="n">
         <v>1</v>
       </c>
@@ -2950,9 +2977,15 @@
       <c r="Q34" t="n">
         <v>1</v>
       </c>
+      <c r="R34" t="n">
+        <v>1</v>
+      </c>
       <c r="S34" t="n">
         <v>1</v>
       </c>
+      <c r="T34" t="n">
+        <v>1</v>
+      </c>
       <c r="U34" t="n">
         <v>1</v>
       </c>
@@ -2960,23 +2993,23 @@
         <v>1</v>
       </c>
       <c r="AF34" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AG34" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH34" t="inlineStr">
         <is>
-          <t>tardio</t>
+          <t>alineado</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Materia y materiales</t>
+          <t>Minerales: composición y estructura cristalina</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2985,71 +3018,35 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F35" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G35" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
-      </c>
-      <c r="I35" t="n">
+        <v>7</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF35" t="n">
         <v>8</v>
       </c>
-      <c r="J35" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K35" t="n">
-        <v>4</v>
-      </c>
-      <c r="L35" t="n">
-        <v>3</v>
-      </c>
-      <c r="M35" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N35" t="n">
-        <v>1</v>
-      </c>
-      <c r="O35" t="n">
-        <v>1</v>
-      </c>
-      <c r="P35" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>1</v>
-      </c>
-      <c r="R35" t="n">
-        <v>1</v>
-      </c>
-      <c r="S35" t="n">
-        <v>1</v>
-      </c>
-      <c r="T35" t="n">
-        <v>1</v>
-      </c>
-      <c r="U35" t="n">
-        <v>1</v>
-      </c>
-      <c r="V35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>2</v>
-      </c>
       <c r="AG35" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH35" t="inlineStr">
@@ -3061,7 +3058,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Minerales: composición y estructura cristalina</t>
+          <t>Modelo de partículas de la materia</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3070,35 +3067,74 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D36" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E36" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F36" t="n">
         <v>8</v>
       </c>
+      <c r="G36" t="n">
+        <v>6</v>
+      </c>
       <c r="H36" t="n">
         <v>7</v>
       </c>
+      <c r="I36" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" t="n">
+        <v>7</v>
+      </c>
+      <c r="K36" t="n">
+        <v>4</v>
+      </c>
+      <c r="L36" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M36" t="n">
+        <v>7</v>
+      </c>
       <c r="N36" t="n">
         <v>1</v>
       </c>
       <c r="O36" t="n">
         <v>1</v>
       </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
       <c r="Q36" t="n">
         <v>1</v>
       </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" t="n">
+        <v>1</v>
+      </c>
+      <c r="T36" t="n">
+        <v>1</v>
+      </c>
+      <c r="U36" t="n">
+        <v>1</v>
+      </c>
+      <c r="V36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>1</v>
+      </c>
       <c r="AF36" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AG36" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>alineado</t>
         </is>
       </c>
       <c r="AH36" t="inlineStr">
@@ -3110,7 +3146,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Modelo de partículas de la materia</t>
+          <t>Compuestos inorgánicos: funciones y nomenclatura</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3119,13 +3155,10 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D37" t="n">
-        <v>6</v>
-      </c>
-      <c r="E37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
         <v>8</v>
@@ -3133,60 +3166,24 @@
       <c r="G37" t="n">
         <v>6</v>
       </c>
-      <c r="H37" t="n">
-        <v>7</v>
-      </c>
-      <c r="I37" t="n">
-        <v>3</v>
-      </c>
-      <c r="J37" t="n">
-        <v>7</v>
-      </c>
-      <c r="K37" t="n">
-        <v>4</v>
-      </c>
-      <c r="L37" t="n">
-        <v>7.5</v>
-      </c>
       <c r="M37" t="n">
         <v>7</v>
       </c>
-      <c r="N37" t="n">
-        <v>1</v>
-      </c>
       <c r="O37" t="n">
         <v>1</v>
       </c>
       <c r="P37" t="n">
         <v>1</v>
       </c>
-      <c r="Q37" t="n">
-        <v>1</v>
-      </c>
-      <c r="R37" t="n">
-        <v>1</v>
-      </c>
-      <c r="S37" t="n">
-        <v>1</v>
-      </c>
-      <c r="T37" t="n">
-        <v>1</v>
-      </c>
-      <c r="U37" t="n">
-        <v>1</v>
-      </c>
       <c r="V37" t="n">
         <v>1</v>
       </c>
-      <c r="Z37" t="n">
-        <v>1</v>
-      </c>
       <c r="AF37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
       <c r="AH37" t="inlineStr">
@@ -6261,7 +6258,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Geometría molecular (RPECV)</t>
+          <t>Fuerzas intermoleculares y propiedades físicas</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -6270,19 +6267,34 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D107" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="F107" t="n">
+        <v>8</v>
       </c>
       <c r="G107" t="n">
         <v>8.5</v>
       </c>
+      <c r="H107" t="n">
+        <v>7</v>
+      </c>
+      <c r="O107" t="n">
+        <v>1</v>
+      </c>
       <c r="P107" t="n">
         <v>1</v>
       </c>
+      <c r="Q107" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z107" t="n">
+        <v>1</v>
+      </c>
       <c r="AF107" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="AG107" t="inlineStr">
         <is>
@@ -6291,14 +6303,14 @@
       </c>
       <c r="AH107" t="inlineStr">
         <is>
-          <t>sin_referente</t>
+          <t>posterior</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Isótopos</t>
+          <t>Geometría molecular (RPECV)</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -6307,25 +6319,19 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D108" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G108" t="n">
         <v>8.5</v>
       </c>
-      <c r="L108" t="n">
-        <v>7.5</v>
-      </c>
       <c r="P108" t="n">
         <v>1</v>
       </c>
-      <c r="U108" t="n">
-        <v>1</v>
-      </c>
       <c r="AF108" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AG108" t="inlineStr">
         <is>
@@ -6341,7 +6347,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Masa molar</t>
+          <t>Isótopos</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -6350,25 +6356,25 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D109" t="n">
-        <v>8</v>
-      </c>
-      <c r="F109" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G109" t="n">
         <v>8.5</v>
       </c>
-      <c r="O109" t="n">
-        <v>1</v>
+      <c r="L109" t="n">
+        <v>7.5</v>
       </c>
       <c r="P109" t="n">
         <v>1</v>
       </c>
+      <c r="U109" t="n">
+        <v>1</v>
+      </c>
       <c r="AF109" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AG109" t="inlineStr">
         <is>
@@ -6384,7 +6390,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Modelo mecanocuántico y orbitales atómicos</t>
+          <t>Masa molar</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6393,13 +6399,25 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D110" t="n">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="F110" t="n">
+        <v>8</v>
+      </c>
+      <c r="G110" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O110" t="n">
+        <v>1</v>
+      </c>
+      <c r="P110" t="n">
+        <v>1</v>
       </c>
       <c r="AF110" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AG110" t="inlineStr">
         <is>
@@ -6415,7 +6433,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Mol y número de Avogadro</t>
+          <t>Modelo mecanocuántico y orbitales atómicos</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6424,25 +6442,13 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D111" t="n">
-        <v>8</v>
-      </c>
-      <c r="F111" t="n">
-        <v>8</v>
-      </c>
-      <c r="G111" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="O111" t="n">
-        <v>1</v>
-      </c>
-      <c r="P111" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF111" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AG111" t="inlineStr">
         <is>
@@ -6458,7 +6464,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Molaridad y unidades químicas de concentración</t>
+          <t>Mol y número de Avogadro</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6472,6 +6478,18 @@
       <c r="D112" t="n">
         <v>8</v>
       </c>
+      <c r="F112" t="n">
+        <v>8</v>
+      </c>
+      <c r="G112" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O112" t="n">
+        <v>1</v>
+      </c>
+      <c r="P112" t="n">
+        <v>1</v>
+      </c>
       <c r="AF112" t="n">
         <v>8</v>
       </c>
@@ -6489,7 +6507,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Compuestos inorgánicos: funciones y nomenclatura</t>
+          <t>Molaridad y unidades químicas de concentración</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6498,31 +6516,13 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D113" t="n">
-        <v>5</v>
-      </c>
-      <c r="F113" t="n">
         <v>8</v>
       </c>
-      <c r="G113" t="n">
-        <v>6</v>
-      </c>
-      <c r="M113" t="n">
-        <v>7</v>
-      </c>
-      <c r="O113" t="n">
-        <v>1</v>
-      </c>
-      <c r="P113" t="n">
-        <v>1</v>
-      </c>
-      <c r="V113" t="n">
-        <v>1</v>
-      </c>
       <c r="AF113" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG113" t="inlineStr">
         <is>
@@ -6531,7 +6531,7 @@
       </c>
       <c r="AH113" t="inlineStr">
         <is>
-          <t>alineado</t>
+          <t>sin_referente</t>
         </is>
       </c>
     </row>

</xml_diff>